<commit_message>
add Login/ Register and Dashboard
</commit_message>
<xml_diff>
--- a/Week_6/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_6/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t>Week_1</t>
   </si>
@@ -177,6 +177,9 @@
   <si>
     <t>Mentor Checklist</t>
   </si>
+  <si>
+    <t>set up the Laravel project, connected the database, installed the login/register system, added user roles (patient, doctor, admin), created role-based dashboard routes, and worked on debugging the login/session issue.</t>
+  </si>
 </sst>
 </file>
 
@@ -323,7 +326,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -476,6 +479,9 @@
     </xf>
     <xf borderId="1" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="10" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="10" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -3083,10 +3089,16 @@
       <c r="AA70" s="3"/>
     </row>
     <row r="71">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
+      <c r="A71" s="49"/>
+      <c r="B71" s="53" t="s">
+        <v>55</v>
+      </c>
+      <c r="C71" s="51">
+        <v>46076.0</v>
+      </c>
+      <c r="D71" s="52">
+        <v>3.75</v>
+      </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -3112,15 +3124,10 @@
       <c r="AA71" s="3"/>
     </row>
     <row r="72">
-      <c r="A72" s="53"/>
-      <c r="B72" s="54" t="s">
-        <v>15</v>
-      </c>
-      <c r="C72" s="55"/>
-      <c r="D72" s="49">
-        <f>sum(D67:D70)</f>
-        <v>5.75</v>
-      </c>
+      <c r="A72" s="3"/>
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
@@ -3146,10 +3153,15 @@
       <c r="AA72" s="3"/>
     </row>
     <row r="73">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
+      <c r="A73" s="54"/>
+      <c r="B73" s="55" t="s">
+        <v>15</v>
+      </c>
+      <c r="C73" s="56"/>
+      <c r="D73" s="49">
+        <f>sum(D67:D71)</f>
+        <v>9.5</v>
+      </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -28694,6 +28706,35 @@
       <c r="Z953" s="3"/>
       <c r="AA953" s="3"/>
     </row>
+    <row r="954">
+      <c r="A954" s="3"/>
+      <c r="B954" s="3"/>
+      <c r="C954" s="3"/>
+      <c r="D954" s="3"/>
+      <c r="E954" s="3"/>
+      <c r="F954" s="3"/>
+      <c r="G954" s="3"/>
+      <c r="H954" s="3"/>
+      <c r="I954" s="3"/>
+      <c r="J954" s="3"/>
+      <c r="K954" s="3"/>
+      <c r="L954" s="3"/>
+      <c r="M954" s="3"/>
+      <c r="N954" s="3"/>
+      <c r="O954" s="3"/>
+      <c r="P954" s="3"/>
+      <c r="Q954" s="3"/>
+      <c r="R954" s="3"/>
+      <c r="S954" s="3"/>
+      <c r="T954" s="3"/>
+      <c r="U954" s="3"/>
+      <c r="V954" s="3"/>
+      <c r="W954" s="3"/>
+      <c r="X954" s="3"/>
+      <c r="Y954" s="3"/>
+      <c r="Z954" s="3"/>
+      <c r="AA954" s="3"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>